<commit_message>
feat: calculate difference in hhsize between surveys
</commit_message>
<xml_diff>
--- a/output/five-decade-tables/compare-surveys - manual edit.xlsx
+++ b/output/five-decade-tables/compare-surveys - manual edit.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ls4540\Documents\dev\households-over-the-years\output\five-decade-tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A53C3D1-0922-4196-A4EE-F4234E691232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C8BCC54-A290-41D4-91A1-3BAD9567CF3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="740" windowWidth="23020" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="compare_surveys" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -83,10 +96,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="175" formatCode="0.0\%"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0\%"/>
+    <numFmt numFmtId="167" formatCode="0.000%"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -129,22 +143,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -446,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.5703125" customWidth="1"/>
@@ -704,6 +721,64 @@
         <v>6.3563882506630906E-2</v>
       </c>
     </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B16">
+        <f>B10/B8</f>
+        <v>1.0130459965464305</v>
+      </c>
+      <c r="C16">
+        <f t="shared" ref="C16:E16" si="0">C10/C8</f>
+        <v>0.99810182643543777</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="0"/>
+        <v>0.98550343342225566</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>0.98018273735570594</v>
+      </c>
+      <c r="F16">
+        <f>F10/F9</f>
+        <v>1.0016153469898053</v>
+      </c>
+      <c r="G16">
+        <f>G10/G9</f>
+        <v>0.98520198809893089</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="5">
+        <f>ABS(B16-1)</f>
+        <v>1.3045996546430461E-2</v>
+      </c>
+      <c r="C17" s="5">
+        <f t="shared" ref="C17:G17" si="1">ABS(C16-1)</f>
+        <v>1.8981735645622333E-3</v>
+      </c>
+      <c r="D17" s="5">
+        <f t="shared" si="1"/>
+        <v>1.4496566577744341E-2</v>
+      </c>
+      <c r="E17" s="5">
+        <f t="shared" si="1"/>
+        <v>1.9817262644294065E-2</v>
+      </c>
+      <c r="F17" s="5">
+        <f t="shared" si="1"/>
+        <v>1.6153469898052553E-3</v>
+      </c>
+      <c r="G17" s="5">
+        <f t="shared" si="1"/>
+        <v>1.4798011901069108E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="G18">
+        <f>G9/B8-1</f>
+        <v>-0.19444446629474632</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>